<commit_message>
novos parsers / coleta das tabelas de resultados finalizadas / inicio montagem xml pt
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO FORTE</t>
+          <t>FPSO-FRADE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231010A-TT</t>
+          <t>044-PT-1020A</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Gás Lift A- Poço ABL-81</t>
+          <t>Oil to Cargo A</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25 - ODS - 70 - TEM - 456</t>
+          <t>25-ODS-37 - PRE - 555</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>22/11/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4519,8 +4519,15 @@
         <is>
           <r>
             <rPr/>
-            <t xml:space="preserve">(  ) Sim ( X ) Não
+            <t xml:space="preserve">( X ) Sim (  ) Não
 OBSERVAÇÕES:
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t xml:space="preserve">Novo range e alarmes alterados no computador de vazão
 </t>
           </r>
         </is>
@@ -4605,7 +4612,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>23/12/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4644,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
inicio validação do código do certificado
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="17565" yWindow="-11370" windowWidth="21600" windowHeight="11175" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet name="Template Formulário" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template Formulário" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Template Formulário'!$A$1:$J$42</definedName>
@@ -385,7 +385,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>5</col>
@@ -405,20 +405,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:xfrm>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:off x="6285122" y="238125"/>
           <a:ext cx="1375503" cy="295882"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
           <avLst/>
         </a:prstGeom>
-        <a:ln>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
extração do n° evaluation
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37 - PRE - 555</t>
+          <t>25-ODS-37-PRE-555</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
ajuste incerteza e tendencia xml petro
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
+          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>044-PT-1020A</t>
+          <t>044-TE-1020A</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37-PRE-555</t>
+          <t>25-ODS-37-TEM-504</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>

</xml_diff>

<commit_message>
implementação da regra de validação dos parametros PO
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO-FRADE</t>
+          <t>FPSO Bravo</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>044-TE-1020A</t>
+          <t>FIT-3115-03</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Oil to Cargo A</t>
+          <t>Gás Combustível</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37-TEM-504</t>
+          <t>26-ODS-53-PRE-016</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>26/01/2026</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>23/12/2025</t>
+          <t>30/01/2026</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
ajuste xml de placa valor angulo borda g
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsmetering-my.sharepoint.com/personal/m_bandeira_odsenergysolutions_com/Documents/Documents/AC's_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D033300120636FCF38C23AD5DA807ADD9E072" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9286378F-5947-48F6-8088-C2B307DD5F1B}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D033300127F5E7FEDFCE1BD5DA807ADD9E020" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63D1BC50-2296-49E0-A1DF-D6B66C70BEC1}"/>
   <bookViews>
     <workbookView xWindow="-15480" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,13 +45,13 @@
     <t>Unidade:</t>
   </si>
   <si>
-    <t>FPSO FRADE</t>
+    <t>ODS LAB</t>
   </si>
   <si>
     <t>Número de série:</t>
   </si>
   <si>
-    <t>ST‐1954‐PO4444‐P01</t>
+    <t>CS-PO-19-11-0147</t>
   </si>
   <si>
     <t>Localização:</t>
@@ -60,13 +60,13 @@
     <t>Número do Certificado:</t>
   </si>
   <si>
-    <t>25‐ODS‐37‐DIM‐022</t>
+    <t>25-ODS-70-DIM-074</t>
   </si>
   <si>
     <t>Data de Calibração:</t>
   </si>
   <si>
-    <t>08/03/2025</t>
+    <t>11/11/2025</t>
   </si>
   <si>
     <t>Empresa Certificadora:</t>
@@ -4242,8 +4242,8 @@
     <col min="6" max="6" width="20.453125" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.1796875" style="1" customWidth="1"/>
     <col min="8" max="9" width="8" style="1" customWidth="1"/>
-    <col min="10" max="12" width="9.1796875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.1796875" style="1"/>
+    <col min="10" max="15" width="9.1796875" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="35.25" customHeight="1">

</xml_diff>

<commit_message>
AC PO - origem
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsmetering-my.sharepoint.com/personal/m_bandeira_odsenergysolutions_com/Documents/Documents/AC's_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D033300127F5E7FEDFCE1BD5DA807ADD9E020" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63D1BC50-2296-49E0-A1DF-D6B66C70BEC1}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D033300122776B085B2E3AC5DA807ADD9E072" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB053ED4-C866-42D6-A19A-775BB45009B0}"/>
   <bookViews>
     <workbookView xWindow="-15480" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,13 +45,13 @@
     <t>Unidade:</t>
   </si>
   <si>
-    <t>ODS LAB</t>
+    <t>FPSO FRADE</t>
   </si>
   <si>
     <t>Número de série:</t>
   </si>
   <si>
-    <t>CS-PO-19-11-0147</t>
+    <t>ST‐1954‐PO4444‐P01</t>
   </si>
   <si>
     <t>Localização:</t>
@@ -60,13 +60,13 @@
     <t>Número do Certificado:</t>
   </si>
   <si>
-    <t>25-ODS-70-DIM-074</t>
+    <t>25‐ODS‐37‐DIM‐022</t>
   </si>
   <si>
     <t>Data de Calibração:</t>
   </si>
   <si>
-    <t>11/11/2025</t>
+    <t>08/03/2025</t>
   </si>
   <si>
     <t>Empresa Certificadora:</t>
@@ -4242,8 +4242,8 @@
     <col min="6" max="6" width="20.453125" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.1796875" style="1" customWidth="1"/>
     <col min="8" max="9" width="8" style="1" customWidth="1"/>
-    <col min="10" max="15" width="9.1796875" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.1796875" style="1"/>
+    <col min="10" max="16" width="9.1796875" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="35.25" customHeight="1">

</xml_diff>

<commit_message>
ajuste extração dos resultados de aprovação Evaluation Rerport Placa
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsmetering-my.sharepoint.com/personal/m_bandeira_odsenergysolutions_com/Documents/Documents/AC's_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D033300122776B085B2E3AC5DA807ADD9E072" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB053ED4-C866-42D6-A19A-775BB45009B0}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D03330012154673F29A60AE5DA807ADD9E072" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52DC07BF-EFE5-42AE-8B31-60C1A9093698}"/>
   <bookViews>
     <workbookView xWindow="-15480" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4242,8 +4242,8 @@
     <col min="6" max="6" width="20.453125" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.1796875" style="1" customWidth="1"/>
     <col min="8" max="9" width="8" style="1" customWidth="1"/>
-    <col min="10" max="16" width="9.1796875" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.1796875" style="1"/>
+    <col min="10" max="17" width="9.1796875" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="35.25" customHeight="1">

</xml_diff>

<commit_message>
ajuste categorização instrumentos diferencial de pressão <= 250 para categorização AC
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão Diferencial</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO FRADE</t>
+          <t>FPSO-FRADE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>041-PDT-9001B</t>
+          <t>070-FT-1006</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>MPMF 9001B - TOPSIDE</t>
+          <t>Fuel Gas</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>26-ODS-37-PRE-106</t>
+          <t>26-ODS-37-PRE-087</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4519,15 +4519,8 @@
         <is>
           <r>
             <rPr/>
-            <t xml:space="preserve">( X ) Sim (  ) Não
+            <t xml:space="preserve">(  ) Sim ( X ) Não
 OBSERVAÇÕES:
-</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="1"/>
-            </rPr>
-            <t xml:space="preserve">Novo range e alarmes alterados no computador de vazão
 </t>
           </r>
         </is>
@@ -4612,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>25/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4644,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
revisão de comentários pastas core/data/form
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="19515" yWindow="-13170" windowWidth="14400" windowHeight="7275" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +82,11 @@
       <b val="1"/>
       <color rgb="FF008080"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Fairwater Script"/>
+      <color theme="1"/>
+      <sz val="20"/>
     </font>
   </fonts>
   <fills count="4">
@@ -233,7 +238,6 @@
   <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -245,7 +249,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -261,6 +264,7 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -307,6 +311,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -730,13 +737,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E143"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="64.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="3.453125" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="13.453125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="3.453125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="50.81640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="64.140625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="3.42578125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="3.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="50.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3980,39 +3987,39 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:J41"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1796875" defaultRowHeight="12"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="12"/>
   <cols>
-    <col width="1.26953125" customWidth="1" style="29" min="1" max="1"/>
-    <col width="23" customWidth="1" style="29" min="2" max="2"/>
-    <col width="22" customWidth="1" style="29" min="3" max="3"/>
-    <col width="18.453125" customWidth="1" style="29" min="4" max="4"/>
-    <col width="23.453125" bestFit="1" customWidth="1" style="29" min="5" max="5"/>
-    <col width="20.453125" customWidth="1" style="29" min="6" max="6"/>
-    <col width="8.1796875" customWidth="1" style="29" min="7" max="7"/>
-    <col width="8" customWidth="1" style="29" min="8" max="9"/>
-    <col width="9.1796875" customWidth="1" style="29" min="10" max="21"/>
-    <col width="9.1796875" customWidth="1" style="29" min="22" max="16384"/>
+    <col width="1.28515625" customWidth="1" style="28" min="1" max="1"/>
+    <col width="23" customWidth="1" style="28" min="2" max="2"/>
+    <col width="22" customWidth="1" style="28" min="3" max="3"/>
+    <col width="18.42578125" customWidth="1" style="28" min="4" max="4"/>
+    <col width="23.42578125" bestFit="1" customWidth="1" style="28" min="5" max="5"/>
+    <col width="20.42578125" customWidth="1" style="28" min="6" max="6"/>
+    <col width="8.140625" customWidth="1" style="28" min="7" max="7"/>
+    <col width="8" customWidth="1" style="28" min="8" max="9"/>
+    <col width="9.140625" customWidth="1" style="28" min="10" max="22"/>
+    <col width="9.140625" customWidth="1" style="28" min="23" max="16384"/>
   </cols>
   <sheetData>
     <row r="2" ht="37.5" customHeight="1">
-      <c r="B2" s="34" t="inlineStr">
+      <c r="B2" s="33" t="inlineStr">
         <is>
           <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="1" t="n"/>
     </row>
     <row r="4" ht="3" customHeight="1">
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="27" t="inlineStr">
         <is>
           <t>Documento Principal: GEN-VAR-PRO-RM-2 - Verificar Metrologicamente Equipamentos de Medição – Sistema de Gestão de Medição (SGM)</t>
         </is>
@@ -4020,502 +4027,502 @@
     </row>
     <row r="5" ht="0.75" customHeight="1"/>
     <row r="6">
-      <c r="B6" s="36" t="n"/>
-      <c r="J6" s="3" t="n"/>
+      <c r="B6" s="35" t="n"/>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Unidade:</t>
         </is>
       </c>
-      <c r="C7" s="35" t="inlineStr">
-        <is>
-          <t>FPSO Bravo</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>FPSO-FRADE</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>TAG do instrumento:</t>
         </is>
       </c>
-      <c r="F7" s="31" t="inlineStr">
-        <is>
-          <t>TIT-3115-52</t>
-        </is>
-      </c>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="n"/>
-      <c r="I7" s="20" t="n"/>
-    </row>
-    <row r="8" ht="14.5" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>044-TT-1020C</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="14.45" customHeight="1">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Localização:</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>Gás Combustível HP</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Oil to Cargo C</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Número do Certificado:</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>26-ODS-53-TEM-111</t>
-        </is>
-      </c>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="19" t="n"/>
-      <c r="I8" s="20" t="n"/>
-    </row>
-    <row r="9" ht="14.5" customHeight="1">
-      <c r="B9" s="6" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>26-0DS-37-TEM-129</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="19" t="n"/>
+    </row>
+    <row r="9" ht="14.45" customHeight="1">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Data de Calibração:</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>03/04/2026</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Empresa Certificadora:</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>ODS Metering Systems</t>
         </is>
       </c>
-      <c r="G9" s="19" t="n"/>
-      <c r="H9" s="19" t="n"/>
-      <c r="I9" s="20" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="19" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1"/>
     <row r="12" ht="12.75" customHeight="1">
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>1.1 Descrição dos itens a serem verificados</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="14.5" customHeight="1">
-      <c r="B13" s="21" t="inlineStr">
+    <row r="13" ht="14.45" customHeight="1">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>a) Identificação unívoca (Número do Certificado de Calibração).</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="14" t="inlineStr">
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H13" s="14" t="n"/>
-      <c r="I13" s="14" t="n"/>
-    </row>
-    <row r="14" ht="14.5" customHeight="1">
-      <c r="B14" s="21" t="inlineStr">
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+    </row>
+    <row r="14" ht="14.45" customHeight="1">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>b) Nome e endereço do Laboratório/Empresa.</t>
         </is>
       </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="19" t="n"/>
-      <c r="F14" s="20" t="n"/>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="C14" s="18" t="n"/>
+      <c r="D14" s="18" t="n"/>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H14" s="14" t="n"/>
-      <c r="I14" s="14" t="n"/>
-    </row>
-    <row r="15" ht="14.5" customHeight="1">
-      <c r="B15" s="21" t="inlineStr">
+      <c r="H14" s="12" t="n"/>
+      <c r="I14" s="12" t="n"/>
+    </row>
+    <row r="15" ht="14.45" customHeight="1">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>c) Logotipo da RBC (para instrumento associado a sistemas de medição fiscal, apropriação, custódia, flare)</t>
         </is>
       </c>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="20" t="n"/>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H15" s="14" t="n"/>
-      <c r="I15" s="14" t="n"/>
-    </row>
-    <row r="16" ht="14.5" customHeight="1">
-      <c r="B16" s="21" t="inlineStr">
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="n"/>
+    </row>
+    <row r="16" ht="14.45" customHeight="1">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>d) Nome e endereço do cliente.</t>
         </is>
       </c>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="20" t="n"/>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H16" s="14" t="n"/>
-      <c r="I16" s="14" t="n"/>
-    </row>
-    <row r="17" ht="14.5" customHeight="1">
-      <c r="B17" s="21" t="inlineStr">
+      <c r="H16" s="12" t="n"/>
+      <c r="I16" s="12" t="n"/>
+    </row>
+    <row r="17" ht="14.45" customHeight="1">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>e) Número de páginas e total de páginas.</t>
         </is>
       </c>
-      <c r="C17" s="19" t="n"/>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="19" t="n"/>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H17" s="14" t="n"/>
-      <c r="I17" s="14" t="n"/>
-    </row>
-    <row r="18" ht="14.5" customHeight="1">
-      <c r="B18" s="21" t="inlineStr">
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="14.45" customHeight="1">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>f) Identificação do método/procedimento utilizado.</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="19" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="C18" s="18" t="n"/>
+      <c r="D18" s="18" t="n"/>
+      <c r="E18" s="18" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H18" s="14" t="n"/>
-      <c r="I18" s="14" t="n"/>
-    </row>
-    <row r="19" ht="14.5" customHeight="1">
-      <c r="B19" s="21" t="inlineStr">
+      <c r="H18" s="12" t="n"/>
+      <c r="I18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="14.45" customHeight="1">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>g) Registro das condições ambientais.</t>
         </is>
       </c>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="20" t="n"/>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H19" s="14" t="n"/>
-      <c r="I19" s="14" t="n"/>
-    </row>
-    <row r="20" ht="14.5" customHeight="1">
-      <c r="B20" s="21" t="inlineStr">
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="14.45" customHeight="1">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>h) Descrição e identificação do item de calibração (ex.: nome, fabricante, tipo, modelo, número de série, etc).</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="20" t="n"/>
-      <c r="G20" s="14" t="inlineStr">
+      <c r="C20" s="18" t="n"/>
+      <c r="D20" s="18" t="n"/>
+      <c r="E20" s="18" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="14" t="n"/>
-    </row>
-    <row r="21" ht="14.5" customHeight="1">
-      <c r="B21" s="21" t="inlineStr">
+      <c r="H20" s="12" t="n"/>
+      <c r="I20" s="12" t="n"/>
+    </row>
+    <row r="21" ht="14.45" customHeight="1">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>i) A data do recebimento do(s) item(s) de calibração, se necessário.</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="20" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
-      <c r="I21" s="14" t="inlineStr">
+      <c r="C21" s="18" t="n"/>
+      <c r="D21" s="18" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="14.5" customHeight="1">
-      <c r="B22" s="21" t="inlineStr">
+    <row r="22" ht="14.45" customHeight="1">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>j) A data da realização da calibração.</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="20" t="n"/>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H22" s="14" t="n"/>
-      <c r="I22" s="14" t="n"/>
-    </row>
-    <row r="23" ht="14.5" customHeight="1">
-      <c r="B23" s="21" t="inlineStr">
+      <c r="H22" s="12" t="n"/>
+      <c r="I22" s="12" t="n"/>
+    </row>
+    <row r="23" ht="14.45" customHeight="1">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>k) Os resultados da calibração estão com as unidades de medida no SI, onde apropriado.</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="20" t="n"/>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="C23" s="18" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H23" s="14" t="n"/>
-      <c r="I23" s="14" t="n"/>
-    </row>
-    <row r="24" ht="14.5" customHeight="1">
-      <c r="B24" s="21" t="inlineStr">
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+    </row>
+    <row r="24" ht="14.45" customHeight="1">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>l) Evidências de que as medições são rastreáveis (Informações dos padrões utilizados).</t>
         </is>
       </c>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-      <c r="E24" s="19" t="n"/>
-      <c r="F24" s="20" t="n"/>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="C24" s="18" t="n"/>
+      <c r="D24" s="18" t="n"/>
+      <c r="E24" s="18" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
+      <c r="H24" s="12" t="n"/>
+      <c r="I24" s="12" t="n"/>
     </row>
     <row r="25" ht="24.75" customHeight="1">
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>m) Nome(s), função (ões) e assinatura (s) ou identificações equivalentes das pessoas autorizadas para emissão do certificado.</t>
         </is>
       </c>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="19" t="n"/>
-      <c r="E25" s="19" t="n"/>
-      <c r="F25" s="20" t="n"/>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="C25" s="18" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-    </row>
-    <row r="26" ht="14.5" customHeight="1">
-      <c r="B26" s="21" t="inlineStr">
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="12" t="n"/>
+    </row>
+    <row r="26" ht="14.45" customHeight="1">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>n) Declaração de que os resultados e incertezas se referem somente aos itens calibrados / inspecionados.</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="19" t="n"/>
-      <c r="F26" s="20" t="n"/>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="C26" s="18" t="n"/>
+      <c r="D26" s="18" t="n"/>
+      <c r="E26" s="18" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H26" s="14" t="n"/>
-      <c r="I26" s="14" t="n"/>
-    </row>
-    <row r="27" ht="14.5" customHeight="1">
-      <c r="B27" s="21" t="inlineStr">
+      <c r="H26" s="12" t="n"/>
+      <c r="I26" s="12" t="n"/>
+    </row>
+    <row r="27" ht="14.45" customHeight="1">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>o) Nível de confiança e fator de abrangência.</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="20" t="n"/>
-      <c r="G27" s="14" t="inlineStr">
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H27" s="14" t="n"/>
-      <c r="I27" s="14" t="n"/>
-    </row>
-    <row r="28" ht="14.5" customHeight="1">
-      <c r="B28" s="21" t="inlineStr">
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+    </row>
+    <row r="28" ht="14.45" customHeight="1">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">p) Foi feita calibração de acordo com a faixa solicitada? </t>
         </is>
       </c>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-      <c r="E28" s="19" t="n"/>
-      <c r="F28" s="20" t="n"/>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="C28" s="18" t="n"/>
+      <c r="D28" s="18" t="n"/>
+      <c r="E28" s="18" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H28" s="14" t="n"/>
-      <c r="I28" s="14" t="n"/>
+      <c r="H28" s="12" t="n"/>
+      <c r="I28" s="12" t="n"/>
     </row>
     <row r="29" ht="24.75" customHeight="1">
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>q) Os erros máximos de medição (Erro sistemático remanescente + incerteza) são inferiores ao erro máximo admissível para o equipamento em questão?</t>
         </is>
       </c>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="19" t="n"/>
-      <c r="E29" s="19" t="n"/>
-      <c r="F29" s="20" t="n"/>
-      <c r="G29" s="14" t="inlineStr">
+      <c r="C29" s="18" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H29" s="14" t="n"/>
-      <c r="I29" s="14" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="12" t="n"/>
     </row>
     <row r="30" ht="25.5" customHeight="1">
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>r) O instrumento está aprovado para o uso no ponto de medição a que se destina de acordo com os critérios de aceitação informados pelo cliente?</t>
         </is>
       </c>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-      <c r="E30" s="19" t="n"/>
-      <c r="F30" s="20" t="n"/>
-      <c r="G30" s="14" t="inlineStr">
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="H30" s="14" t="n"/>
-      <c r="I30" s="14" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
     </row>
     <row r="31" ht="25.5" customHeight="1">
-      <c r="B31" s="21" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>s) No caso de ajuste no equipamento, estão informados os resultados das calibrações como encontrados (as found) e como deixados (as left)?</t>
         </is>
       </c>
-      <c r="C31" s="19" t="n"/>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="19" t="n"/>
-      <c r="F31" s="20" t="n"/>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="14" t="n"/>
-      <c r="I31" s="14" t="inlineStr">
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
     </row>
     <row r="32" ht="27" customHeight="1">
-      <c r="B32" s="32" t="inlineStr">
+      <c r="B32" s="31" t="inlineStr">
         <is>
           <t>1.2 É recomendado que o relatório de análise contenha uma declaração especificando que o mesmo só deve ser reproduzido completo.  Reprodução de partes requer aprovação escrita do emitente. O relatório apresentado atende esta recomendação?</t>
         </is>
       </c>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="19" t="n"/>
-      <c r="F32" s="19" t="n"/>
-      <c r="G32" s="19" t="n"/>
-      <c r="H32" s="19" t="n"/>
-      <c r="I32" s="20" t="n"/>
+      <c r="C32" s="18" t="n"/>
+      <c r="D32" s="18" t="n"/>
+      <c r="E32" s="18" t="n"/>
+      <c r="F32" s="18" t="n"/>
+      <c r="G32" s="18" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="19" t="n"/>
     </row>
     <row r="33" ht="66.75" customHeight="1">
-      <c r="B33" s="30" t="inlineStr">
+      <c r="B33" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">( X )   Sim      (   ) Não
 OBSERVAÇÕES:
 </t>
         </is>
       </c>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="19" t="n"/>
-      <c r="F33" s="19" t="n"/>
-      <c r="G33" s="19" t="n"/>
-      <c r="H33" s="19" t="n"/>
-      <c r="I33" s="20" t="n"/>
+      <c r="C33" s="18" t="n"/>
+      <c r="D33" s="18" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="18" t="n"/>
+      <c r="H33" s="18" t="n"/>
+      <c r="I33" s="19" t="n"/>
     </row>
     <row r="34" ht="30.75" customHeight="1">
-      <c r="B34" s="32" t="inlineStr">
+      <c r="B34" s="31" t="inlineStr">
         <is>
           <t>1.3 Existe alguma informação no documento analisado que necessite ser atualizada em algum outro dispositivo (ex.: range de calibração no computador de vazão)?</t>
         </is>
       </c>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="19" t="n"/>
-      <c r="F34" s="19" t="n"/>
-      <c r="G34" s="19" t="n"/>
-      <c r="H34" s="19" t="n"/>
-      <c r="I34" s="20" t="n"/>
+      <c r="C34" s="18" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="18" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="19" t="n"/>
     </row>
     <row r="35" ht="77.25" customHeight="1">
-      <c r="B35" s="30" t="inlineStr">
+      <c r="B35" s="29" t="inlineStr">
         <is>
           <r>
             <rPr/>
@@ -4525,111 +4532,116 @@
           </r>
         </is>
       </c>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="19" t="n"/>
-      <c r="F35" s="19" t="n"/>
-      <c r="G35" s="19" t="n"/>
-      <c r="H35" s="19" t="n"/>
-      <c r="I35" s="20" t="n"/>
+      <c r="C35" s="18" t="n"/>
+      <c r="D35" s="18" t="n"/>
+      <c r="E35" s="18" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="19" t="n"/>
     </row>
     <row r="36" ht="27.75" customHeight="1">
-      <c r="B36" s="32" t="inlineStr">
+      <c r="B36" s="31" t="inlineStr">
         <is>
           <t>1.4 De acordo com a data do último ensaio / análise que foi realizada no equipamento / produto, observando a periodicidade estabelecida para realização do mesmo; a periodicidade de realização foi cumprida?</t>
         </is>
       </c>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="19" t="n"/>
-      <c r="E36" s="19" t="n"/>
-      <c r="F36" s="19" t="n"/>
-      <c r="G36" s="19" t="n"/>
-      <c r="H36" s="19" t="n"/>
-      <c r="I36" s="20" t="n"/>
+      <c r="C36" s="18" t="n"/>
+      <c r="D36" s="18" t="n"/>
+      <c r="E36" s="18" t="n"/>
+      <c r="F36" s="18" t="n"/>
+      <c r="G36" s="18" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="19" t="n"/>
     </row>
     <row r="37" ht="63.75" customHeight="1">
-      <c r="B37" s="33" t="inlineStr">
+      <c r="B37" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">(   X   )  Sim       (      ) Não
 OBSERVAÇÕES: </t>
         </is>
       </c>
-      <c r="C37" s="19" t="n"/>
-      <c r="D37" s="19" t="n"/>
-      <c r="E37" s="19" t="n"/>
-      <c r="F37" s="19" t="n"/>
-      <c r="G37" s="19" t="n"/>
-      <c r="H37" s="19" t="n"/>
-      <c r="I37" s="20" t="n"/>
+      <c r="C37" s="18" t="n"/>
+      <c r="D37" s="18" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="18" t="n"/>
+      <c r="H37" s="18" t="n"/>
+      <c r="I37" s="19" t="n"/>
     </row>
     <row r="38" ht="28.5" customHeight="1">
-      <c r="B38" s="32" t="inlineStr">
+      <c r="B38" s="31" t="inlineStr">
         <is>
           <t>1.5 Conclusão da análise crítica do relatório de calibração.
 O certificado está conforme requerimento do cliente e RTM?</t>
         </is>
       </c>
-      <c r="C38" s="19" t="n"/>
-      <c r="D38" s="19" t="n"/>
-      <c r="E38" s="19" t="n"/>
-      <c r="F38" s="19" t="n"/>
-      <c r="G38" s="19" t="n"/>
-      <c r="H38" s="19" t="n"/>
-      <c r="I38" s="20" t="n"/>
+      <c r="C38" s="18" t="n"/>
+      <c r="D38" s="18" t="n"/>
+      <c r="E38" s="18" t="n"/>
+      <c r="F38" s="18" t="n"/>
+      <c r="G38" s="18" t="n"/>
+      <c r="H38" s="18" t="n"/>
+      <c r="I38" s="19" t="n"/>
     </row>
     <row r="39" ht="64.5" customHeight="1">
-      <c r="B39" s="23" t="inlineStr">
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>(   X   )  Sim       (      ) Não*
 *Caso a resposta seja “Não”, justifique:</t>
         </is>
       </c>
-      <c r="C39" s="24" t="n"/>
-      <c r="D39" s="24" t="n"/>
-      <c r="E39" s="24" t="n"/>
-      <c r="F39" s="24" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="24" t="n"/>
-      <c r="I39" s="25" t="n"/>
+      <c r="C39" s="23" t="n"/>
+      <c r="D39" s="23" t="n"/>
+      <c r="E39" s="23" t="n"/>
+      <c r="F39" s="23" t="n"/>
+      <c r="G39" s="23" t="n"/>
+      <c r="H39" s="23" t="n"/>
+      <c r="I39" s="24" t="n"/>
     </row>
     <row r="40" ht="33" customHeight="1">
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="12" t="n"/>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="13" t="inlineStr">
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="36" t="inlineStr">
+        <is>
+          <t>Carolina Bastos</t>
+        </is>
+      </c>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="11" t="inlineStr">
         <is>
           <t>Data:</t>
         </is>
       </c>
-      <c r="G40" s="15" t="n"/>
-      <c r="H40" s="17" t="inlineStr">
-        <is>
-          <t>09/04/2026</t>
-        </is>
-      </c>
-      <c r="I40" s="16" t="n"/>
+      <c r="G40" s="13" t="n"/>
+      <c r="H40" s="15" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="I40" s="14" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
-      <c r="B41" s="9" t="n"/>
-      <c r="C41" s="10" t="n"/>
-      <c r="D41" s="27" t="inlineStr">
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="9" t="n"/>
+      <c r="D41" s="26" t="inlineStr">
         <is>
           <t>Responsável pela análise</t>
         </is>
       </c>
-      <c r="E41" s="19" t="n"/>
-      <c r="F41" s="10" t="n"/>
-      <c r="G41" s="10" t="n"/>
-      <c r="H41" s="10" t="n"/>
-      <c r="I41" s="11" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" s="10" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="39">
     <mergeCell ref="F9:I9"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="B31:F31"/>
+    <mergeCell ref="D40:E40"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B27:F27"/>

</xml_diff>

<commit_message>
ajuste xml parâmetros de incerteza e desvio - trasmissor pressão saída eletrica para kPa
</commit_message>
<xml_diff>
--- a/TemplateAC_PRIO.xlsx
+++ b/TemplateAC_PRIO.xlsx
@@ -4004,7 +4004,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="33" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>FPSO-FRADE</t>
+          <t>FPSO Bravo</t>
         </is>
       </c>
       <c r="D7" s="19" t="n"/>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="F7" s="30" t="inlineStr">
         <is>
-          <t>044-TT-1020C</t>
+          <t>PIT-1198B-61</t>
         </is>
       </c>
       <c r="G7" s="18" t="n"/>
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>Oil to Cargo C</t>
+          <t>Tramo B</t>
         </is>
       </c>
       <c r="D8" s="19" t="n"/>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>26-0DS-37-TEM-129</t>
+          <t>26-ODS-53-PRE-076</t>
         </is>
       </c>
       <c r="G8" s="18" t="n"/>
@@ -4090,7 +4090,7 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D9" s="19" t="n"/>
@@ -4616,7 +4616,7 @@
       <c r="G40" s="13" t="n"/>
       <c r="H40" s="15" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>06/03/2026</t>
         </is>
       </c>
       <c r="I40" s="14" t="n"/>

</xml_diff>